<commit_message>
Added new RDF data schemes and visual schemes for economy-table45-49
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table49.xlsx
+++ b/sources/table_normalization/xlsx/economy-table49.xlsx
@@ -202,9 +202,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -215,6 +212,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -529,7 +529,7 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="5">
+      <c r="A2" s="9">
         <v>142</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -558,7 +558,7 @@
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="5"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -579,7 +579,7 @@
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="5"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -600,7 +600,7 @@
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="3"/>
@@ -619,7 +619,7 @@
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="5">
+      <c r="A6" s="9">
         <v>144</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -648,7 +648,7 @@
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="5"/>
+      <c r="A7" s="9"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -669,7 +669,7 @@
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="5"/>
+      <c r="A8" s="9"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -690,7 +690,7 @@
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="5"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -711,7 +711,7 @@
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="3"/>
@@ -730,7 +730,7 @@
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="5">
+      <c r="A11" s="9">
         <v>145</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -759,7 +759,7 @@
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="5"/>
+      <c r="A12" s="9"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -780,7 +780,7 @@
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="3"/>
@@ -828,7 +828,7 @@
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="3"/>
@@ -847,7 +847,7 @@
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="5">
+      <c r="A16" s="9">
         <v>147</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -876,7 +876,7 @@
       </c>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="5"/>
+      <c r="A17" s="9"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -897,7 +897,7 @@
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>25</v>
       </c>
       <c r="B18" s="3"/>
@@ -916,21 +916,21 @@
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="8">
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="7">
         <v>4596</v>
       </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8">
+      <c r="G19" s="7"/>
+      <c r="H19" s="7">
         <v>65917.119999999995</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="7">
         <v>94080.75</v>
       </c>
     </row>

</xml_diff>